<commit_message>
update committees and link
</commit_message>
<xml_diff>
--- a/about/Leadership_2025-26.xlsx
+++ b/about/Leadership_2025-26.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10928"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11122"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/emma/docs/apls-org/about/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B756D56C-D13B-8543-BC52-DE398435FD3B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DAEB448B-AFC7-8245-8129-75E85C29D577}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2900" yWindow="560" windowWidth="38680" windowHeight="13860" firstSheet="7" activeTab="26" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2900" yWindow="560" windowWidth="16900" windowHeight="13320" firstSheet="19" activeTab="26" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="EC" sheetId="1" r:id="rId1"/>
@@ -2153,8 +2153,8 @@
       <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
-        <v>377</v>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
       </c>
       <c r="C1" t="s">
         <v>2</v>
@@ -2240,8 +2240,8 @@
       <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
-        <v>377</v>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
       </c>
       <c r="C1" t="s">
         <v>2</v>
@@ -2372,8 +2372,8 @@
       <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
-        <v>377</v>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
       </c>
       <c r="C1" t="s">
         <v>2</v>
@@ -2461,8 +2461,8 @@
       <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
-        <v>377</v>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
       </c>
       <c r="C1" t="s">
         <v>2</v>
@@ -2620,8 +2620,8 @@
       <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
-        <v>377</v>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
       </c>
       <c r="C1" t="s">
         <v>2</v>
@@ -2798,8 +2798,8 @@
       <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
-        <v>377</v>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
       </c>
       <c r="C1" t="s">
         <v>2</v>
@@ -2901,8 +2901,8 @@
       <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
-        <v>377</v>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
       </c>
       <c r="C1" t="s">
         <v>2</v>
@@ -3093,8 +3093,8 @@
       <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
-        <v>377</v>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
       </c>
       <c r="C1" t="s">
         <v>2</v>
@@ -3256,8 +3256,8 @@
       <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
-        <v>377</v>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
       </c>
       <c r="C1" t="s">
         <v>2</v>
@@ -3336,8 +3336,8 @@
       <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
-        <v>377</v>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
       </c>
       <c r="C1" t="s">
         <v>2</v>
@@ -3662,8 +3662,8 @@
       <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
-        <v>377</v>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
       </c>
       <c r="C1" t="s">
         <v>2</v>
@@ -3995,6 +3995,7 @@
     <row r="22" spans="1:10" ht="16" customHeight="1"/>
   </sheetData>
   <mergeCells count="17">
+    <mergeCell ref="I8:J8"/>
     <mergeCell ref="I15:J15"/>
     <mergeCell ref="I16:J16"/>
     <mergeCell ref="I17:J17"/>
@@ -4011,7 +4012,6 @@
     <mergeCell ref="I5:J5"/>
     <mergeCell ref="I6:J6"/>
     <mergeCell ref="I7:J7"/>
-    <mergeCell ref="I8:J8"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="C2" r:id="rId1" xr:uid="{8E7A33AC-1B97-2A44-8663-826F3172ADED}"/>
@@ -4032,8 +4032,8 @@
       <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
-        <v>377</v>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
       </c>
       <c r="C1" t="s">
         <v>2</v>
@@ -4104,8 +4104,8 @@
       <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
-        <v>377</v>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
       </c>
       <c r="C1" t="s">
         <v>2</v>
@@ -4162,8 +4162,8 @@
       <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
-        <v>377</v>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
       </c>
       <c r="C1" t="s">
         <v>2</v>
@@ -4343,8 +4343,8 @@
       <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
-        <v>377</v>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
       </c>
       <c r="C1" t="s">
         <v>2</v>
@@ -4607,8 +4607,8 @@
       <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
-        <v>377</v>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
       </c>
       <c r="C1" t="s">
         <v>2</v>
@@ -4698,8 +4698,8 @@
       <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
-        <v>377</v>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
       </c>
       <c r="C1" t="s">
         <v>2</v>
@@ -5024,8 +5024,8 @@
       <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
-        <v>377</v>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
       </c>
       <c r="C1" t="s">
         <v>2</v>
@@ -5316,8 +5316,8 @@
       <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
-        <v>377</v>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
       </c>
       <c r="C1" t="s">
         <v>2</v>

</xml_diff>